<commit_message>
集群调度新增Atlas 950 SuperPoD Flex 支持
Co-authored-by: leon_xun<xunzeliang@h-partners.com>
</commit_message>
<xml_diff>
--- a/docs/zh/resource/数据信息说明.xlsx
+++ b/docs/zh/resource/数据信息说明.xlsx
@@ -102,7 +102,8 @@
 Atlas 350 加速卡
 Atlas 850E 超节点
 Atlas 650E 服务器
-Atlas 950 SuperPoD 超节点</t>
+Atlas 950 SuperPoD 超节点
+Atlas 950 SuperPoD Flex</t>
   </si>
   <si>
     <t>nodeBase</t>
@@ -326,7 +327,8 @@
     <t>Atlas 350 加速卡（4Pmesh互联）
 Atlas 850E 超节点
 Atlas 650E 服务器
-Atlas 950 SuperPoD 超节点</t>
+Atlas 950 SuperPoD 超节点
+Atlas 950 SuperPoD Flex</t>
   </si>
   <si>
     <r>
@@ -672,6 +674,7 @@
 Atlas 850E 超节点
 Atlas 650E 服务器
 Atlas 950 SuperPoD 超节点
+Atlas 950 SuperPoD Flex
 说明：
 只有Atlas 推理系列产品为板卡功耗，其余产品为</t>
     </r>
@@ -767,7 +770,8 @@
 Atlas 350 加速卡
 Atlas 850E 超节点
 Atlas 650E 服务器
-Atlas 950 SuperPoD 超节点</t>
+Atlas 950 SuperPoD 超节点
+Atlas 950 SuperPoD Flex</t>
   </si>
   <si>
     <t>container_npu_used_memory</t>
@@ -868,7 +872,8 @@
 Atlas 350 加速卡
 Atlas 850E 超节点
 Atlas 650E 服务器
-Atlas 950 SuperPoD 超节点</t>
+Atlas 950 SuperPoD 超节点
+Atlas 950 SuperPoD Flex</t>
   </si>
   <si>
     <t>npu_chip_info_vector_utilization</t>
@@ -903,7 +908,8 @@
 Atlas 350 加速卡
 Atlas 850E 超节点
 Atlas 650E 服务器
-Atlas 950 SuperPoD 超节点</t>
+Atlas 950 SuperPoD 超节点
+Atlas 950 SuperPoD Flex</t>
   </si>
   <si>
     <t>RoCE</t>
@@ -992,7 +998,8 @@
 Atlas 350 加速卡
 Atlas 850E 超节点
 Atlas 650E 服务器
-Atlas 950 SuperPoD 超节点</t>
+Atlas 950 SuperPoD 超节点
+Atlas 950 SuperPoD Flex</t>
   </si>
   <si>
     <t>npu_chip_info_hbm_total_memory</t>
@@ -1346,7 +1353,8 @@
 Atlas 350 加速卡
 Atlas 850E 超节点
 Atlas 650E 服务器
-Atlas 950 SuperPoD 超节点</t>
+Atlas 950 SuperPoD 超节点
+Atlas 950 SuperPoD Flex</t>
   </si>
   <si>
     <t>npu_chip_info_sio_crc_rx_err_cnt</t>

</xml_diff>